<commit_message>
chore(tm): roll out the all-on v3.5 records (37+3 deliverables, evidence 0008-0011)
</commit_message>
<xml_diff>
--- a/协作/02-任务切片图.xlsx
+++ b/协作/02-任务切片图.xlsx
@@ -607,10 +607,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="只能选择下拉里的值" type="list">
+    <dataValidation sqref="G2:G121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"待派工,进行中,审查中,验证中,集成中,已完成,阻塞"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="只能选择下拉里的值" type="list">
+    <dataValidation sqref="H2:H121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"负责人,产品,需求分析,架构契约,实现工程师,代码评审,专项评审,测试验证,集成发布"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
chore(tm): move the protocol and templates to the TEAMODEL repo, DCG keeps only its own records
</commit_message>
<xml_diff>
--- a/协作/02-任务切片图.xlsx
+++ b/协作/02-任务切片图.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -602,6 +602,53 @@
       <c r="I3" t="inlineStr">
         <is>
           <t>2 小时</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>切片-0004</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>把协议与模板迁出 DCG，改由 TEAMODEL 仓库按标签引用</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TEAMODEL.md;协作/模板/**;docs/TEAMODEL_draft_v1.md;协作/**（仅记录）</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>dcg/**;tests/**;evidence/**;bench/**;CONTRACT.md;DESIGN.md;README.md;pyproject.toml</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>切片-0003</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>guozhizhuang</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>约 1 小时</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(tm): record slice-0005 (README rewrite) with evidence-0014
</commit_message>
<xml_diff>
--- a/协作/02-任务切片图.xlsx
+++ b/协作/02-任务切片图.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -649,6 +649,53 @@
       <c r="I4" t="inlineStr">
         <is>
           <t>约 1 小时</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>切片-0005</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>README 去掉 v2 版本叙事，把「定位」改为适配场景</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>dcg/**;tests/**;evidence/**;bench/**;CONTRACT.md;DESIGN.md;pyproject.toml;协作/**（仅记录）</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>切片-0004</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>guozhizhuang</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>约 30 分钟</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(tm): record slice-0006 (README positioning) with evidence-0015
</commit_message>
<xml_diff>
--- a/协作/02-任务切片图.xlsx
+++ b/协作/02-任务切片图.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -696,6 +696,53 @@
       <c r="I5" t="inlineStr">
         <is>
           <t>约 30 分钟</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>切片-0006</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>README 写明：JSONata 是结构描述语言、编译成固化 Python 提效、主场景为任意数据结构转换</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>dcg/**;tests/**;evidence/**;bench/**;CONTRACT.md;DESIGN.md;pyproject.toml;协作/**（仅记录）</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>切片-0005</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>guozhizhuang</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>约 20 分钟</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(tm): record slice-0007 (README trims) with evidence-0016
</commit_message>
<xml_diff>
--- a/协作/02-任务切片图.xlsx
+++ b/协作/02-任务切片图.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -743,6 +743,53 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>约 20 分钟</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>切片-0007</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>README 删除基线/修订锚点段与 §0.1–§0.3 三个子节，§0 只保留主场景</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>dcg/**;tests/**;evidence/**;bench/**;CONTRACT.md;DESIGN.md;pyproject.toml;协作/**（仅记录）</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>切片-0006</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>guozhizhuang</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>约 15 分钟</t>
         </is>
       </c>
     </row>

</xml_diff>